<commit_message>
fix CSP and event listener
</commit_message>
<xml_diff>
--- a/drugs.xlsx
+++ b/drugs.xlsx
@@ -5,19 +5,21 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\masah\Documents\お薬手帳読み取り\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\masah\drug-check-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C65FABB-41BC-49ED-94FE-1ACD27BD6743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4071665-E1A9-4227-B37E-9253F6F2B50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{2CDA0925-413E-497E-8611-272C1BE2567D}"/>
   </bookViews>
   <sheets>
-    <sheet name="全薬剤" sheetId="1" r:id="rId1"/>
+    <sheet name="休薬一覧" sheetId="1" r:id="rId1"/>
+    <sheet name="配合錠一覧" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">全薬剤!$A$1:$G$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">全薬剤!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">休薬一覧!$A$1:$G$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">配合錠一覧!$A$1:$F$84</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">休薬一覧!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1374" uniqueCount="529">
   <si>
     <t>薬効分類</t>
     <rPh sb="0" eb="4">
@@ -1836,6 +1838,1257 @@
     <t>休薬期間</t>
     <rPh sb="0" eb="4">
       <t>キュウヤクキカン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エゼチミブ錠10mg　１錠</t>
+    <rPh sb="12" eb="13">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロスバスタチンOD錠2.5mg　１錠</t>
+    <rPh sb="17" eb="18">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エゼチミブ10mg</t>
+  </si>
+  <si>
+    <t>ロスバスタチン2.5mg</t>
+  </si>
+  <si>
+    <t>脂異：スタチン＋ゼチーア</t>
+    <rPh sb="0" eb="1">
+      <t>アブラ</t>
+    </rPh>
+    <rPh sb="1" eb="2">
+      <t>イ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロスーゼット配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロスバスタチンOD錠5mg　１錠</t>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロスバスタチン5mg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロスーゼット配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ヒドロクロロチアジド錠12.5mg　１錠</t>
+    <rPh sb="19" eb="20">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロサルタンK錠25mg　２錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ヒドロクロロチアジド12.5mg</t>
+  </si>
+  <si>
+    <t>ロサルタン50mg</t>
+  </si>
+  <si>
+    <t>降圧剤：ARB+利尿剤</t>
+    <rPh sb="0" eb="3">
+      <t>コウアツザイ</t>
+    </rPh>
+    <rPh sb="8" eb="11">
+      <t>リニョウザイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロサルヒド配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロサルタンK錠25mg　４錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロサルタン100mg</t>
+  </si>
+  <si>
+    <t>ロサルヒド配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アゼルニジピン錠16mg　0.5錠</t>
+    <rPh sb="16" eb="17">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>オルメサルタンOD錠10mg　１錠</t>
+    <rPh sb="16" eb="17">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アゼルニジピン８mg</t>
+  </si>
+  <si>
+    <t>オルメサルタン１０mg</t>
+  </si>
+  <si>
+    <t>降圧剤：ARB+CaB</t>
+    <rPh sb="0" eb="3">
+      <t>コウアツザイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>レザルタス配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アゼルニジピン錠16mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>オルメサルタンOD錠20mg　１錠</t>
+    <rPh sb="16" eb="17">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アゼルニジピン１６mg</t>
+  </si>
+  <si>
+    <t>オルメサルタン２０mg</t>
+  </si>
+  <si>
+    <t>レザルタス配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ピタバスタチンカルシウムOD錠2mg　1錠</t>
+    <rPh sb="20" eb="21">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ピタバスタチン2mg</t>
+  </si>
+  <si>
+    <t>リバゼブ配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ピタバスタチンカルシウムOD錠2mg　２錠</t>
+    <rPh sb="20" eb="21">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ピタバスタチン4mg</t>
+  </si>
+  <si>
+    <t>リバゼブ配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ピオグリタゾンOD錠15mg　１錠</t>
+    <rPh sb="16" eb="17">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>採用なし</t>
+    <rPh sb="0" eb="2">
+      <t>サイヨウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ピオグリタゾン15mg</t>
+  </si>
+  <si>
+    <t>アログリプチン25mg</t>
+  </si>
+  <si>
+    <t>糖尿病：TZD+DPP-４</t>
+    <rPh sb="0" eb="3">
+      <t>トウニョウビョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>リオベル配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ピオグリタゾンOD錠15mg　２錠</t>
+    <rPh sb="16" eb="17">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ピオグリタゾン30mg</t>
+  </si>
+  <si>
+    <t>リオベル配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムロジピンOD錠2.5mg　１錠</t>
+    <rPh sb="16" eb="17">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カンデサルタン錠4mg　２錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムロジピンOD錠2.5mg</t>
+  </si>
+  <si>
+    <t>カンデサルタン８mg</t>
+  </si>
+  <si>
+    <t>ユニシア配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムロジピンOD錠5mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムロジピンOD錠５mg</t>
+  </si>
+  <si>
+    <t>ユニシア配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ビルダグリプチン50mg　１錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メトグルコ錠250mg　１錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ビルダグリプチン50mg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メトホルミン25０mg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>糖尿病：BG+DPP-４</t>
+    <rPh sb="0" eb="3">
+      <t>トウニョウビョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メホビル配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ビルダグリプチン50mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メトグルコ錠250mg　２錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メトホルミン5０0mg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メホビル配合錠HＤ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アナグリプチン100mg</t>
+  </si>
+  <si>
+    <t>メトアナ配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メトホルミン５００mg</t>
+  </si>
+  <si>
+    <t>メトアナ配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>糖尿病：BG+TZD</t>
+    <rPh sb="0" eb="3">
+      <t>トウニョウビョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メタクト配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>メタクト配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ヒドロクロロチアジド錠12.5mg　１錠</t>
+    <rPh sb="10" eb="11">
+      <t>ジョウ</t>
+    </rPh>
+    <rPh sb="19" eb="20">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>テルミサルタン２０mg　4錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ヒドロクロロチアジド１2.5mg</t>
+  </si>
+  <si>
+    <t>テルミサルタン8０mg</t>
+  </si>
+  <si>
+    <t>ミコンビ配合錠BＰ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>テルミサルタン２０mg　2錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>テルミサルタン４０mg</t>
+  </si>
+  <si>
+    <t>ミコンビ配合錠ＡＰ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムロジピンOD錠5mg　１錠</t>
+    <rPh sb="8" eb="9">
+      <t>ジョウ</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ミカムロ配合錠BＰ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ミカムロ配合錠ＡＰ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ヒドロクロロチアジド錠12.5mg　１錠
+アムロジピンOD錠5mg　１錠</t>
+    <rPh sb="10" eb="11">
+      <t>ジョウ</t>
+    </rPh>
+    <rPh sb="19" eb="20">
+      <t>ジョウ</t>
+    </rPh>
+    <rPh sb="35" eb="36">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ヒドロクロロチアジド１2.5mg
+アムロジピンOD錠５mg</t>
+  </si>
+  <si>
+    <t>降圧剤：ARB+CaB+利尿剤</t>
+    <rPh sb="0" eb="3">
+      <t>コウアツザイ</t>
+    </rPh>
+    <rPh sb="12" eb="15">
+      <t>リニョウザイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ミカトリオ配合錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>プレミネント配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>プレミネント配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ヒドロクロロチアジド錠12.5mg　0.5錠</t>
+    <rPh sb="21" eb="22">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ヒドロクロロチアジド6.25mg</t>
+  </si>
+  <si>
+    <t>バルサルタン80mg</t>
+  </si>
+  <si>
+    <t>バルヒディオ配合錠MD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>バルヒディオ配合錠EX</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ジャディアンス錠10mg　2.5錠</t>
+    <rPh sb="16" eb="17">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>トラゼンタ錠5mg　１錠</t>
+    <rPh sb="11" eb="12">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エンパグリフロジン２5mg</t>
+  </si>
+  <si>
+    <t>リナグリプチン5mg</t>
+  </si>
+  <si>
+    <t>糖尿病：SGLT2+DPP-４</t>
+    <rPh sb="0" eb="3">
+      <t>トウニョウビョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>トラディアンス配合錠BP</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ジャディアンス錠10mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エンパグリフロジン10mg</t>
+  </si>
+  <si>
+    <t>トラディアンス配合錠AP</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>テルチア配合錠BＰ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>テルチア配合錠ＡＰ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>テラムロ配合錠ＢＰ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>テラムロ配合錠AP</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ランソプラゾールOD錠15mg　１錠</t>
+    <rPh sb="17" eb="18">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>バイアスピリン錠100mg　1錠</t>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ランソプラゾール15mg</t>
+  </si>
+  <si>
+    <t>アスピリン錠100mg</t>
+    <rPh sb="5" eb="6">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>循環器：アスピリン＋胃薬</t>
+    <rPh sb="0" eb="3">
+      <t>ジュンカンキ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>イグスリ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タケルダ配合錠</t>
+    <rPh sb="4" eb="7">
+      <t>ハイゴウジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>グリメピリドOD錠1mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>グリメピリド1mg</t>
+  </si>
+  <si>
+    <t>糖尿病：TZD+SU</t>
+    <rPh sb="0" eb="3">
+      <t>トウニョウビョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ソニアス配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>グリメピリドOD錠1mg　３錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>グリメピリド3mg</t>
+  </si>
+  <si>
+    <t>ソニアス配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ジャヌビア錠50mg　１錠</t>
+    <rPh sb="12" eb="13">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>イプラグリフロジン５０mg</t>
+  </si>
+  <si>
+    <t>シタグリプチン50mg</t>
+  </si>
+  <si>
+    <t>スージャヌ配合錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アジルサルタン錠20mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アジルサルタン２０mg</t>
+  </si>
+  <si>
+    <t>ジルムロ配合錠LＤ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ジルムロ配合錠ＨＤ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ザクラス配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ザクラス配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>クロピドグレル錠75mg　1錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>クロピドグレル75mg</t>
+  </si>
+  <si>
+    <t>コンプラビン配合錠</t>
+    <rPh sb="6" eb="9">
+      <t>ハイゴウジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>コディオ配合錠MD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>コディオ配合錠EX</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ボグリボースOD錠0.2mg　１錠</t>
+    <rPh sb="16" eb="17">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>グルファスト錠10mg　１錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ボグリボース0.2mg</t>
+  </si>
+  <si>
+    <t>ミチグリニド１０mg</t>
+  </si>
+  <si>
+    <t>糖尿病：グリニド+α-GI</t>
+    <rPh sb="0" eb="3">
+      <t>トウニョウビョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>グルベス配合錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タケキャブOD錠10mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ボノプラザン10mg</t>
+  </si>
+  <si>
+    <t>キャプビリン配合錠</t>
+    <rPh sb="6" eb="9">
+      <t>ハイゴウジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カムシア配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カムシア配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カナグルOD錠100mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>テネリアOD錠20mg　１錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カナグリフロジン100mg</t>
+  </si>
+  <si>
+    <t>テネリグリプチン２０mg</t>
+  </si>
+  <si>
+    <t>カナリア配合錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン錠10mg　１錠</t>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムロジピンOD錠５mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン10mg</t>
+  </si>
+  <si>
+    <t>降圧剤：CaB+スタチン</t>
+    <rPh sb="0" eb="3">
+      <t>コウアツザイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カデュエット配合錠４番</t>
+    <rPh sb="10" eb="11">
+      <t>バン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン錠5mg　１錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン5mg</t>
+  </si>
+  <si>
+    <t>カデュエット配合錠３番</t>
+    <rPh sb="10" eb="11">
+      <t>バン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カデュエット配合錠２番</t>
+    <rPh sb="10" eb="11">
+      <t>バン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カデュエット配合錠１番</t>
+    <rPh sb="10" eb="11">
+      <t>バン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カンデサルタン錠4mg　１錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カンデサルタン４mg</t>
+  </si>
+  <si>
+    <t>カデチア配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>カンデサルタン8mg</t>
+  </si>
+  <si>
+    <t>カデチア配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エックスフォージ配合錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ロスバスタチン2.5mg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エゼロス配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エゼロス配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン錠10mg　1錠</t>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン1０mg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エゼアト配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン錠10mg　2錠</t>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン2０mg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エゼアト配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ビルダグリプリン錠50mg　１錠</t>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ビルダグリプチン５０mg</t>
+  </si>
+  <si>
+    <t>メトホルミン250mg</t>
+  </si>
+  <si>
+    <t>エクメット配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エクメット配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エカード配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>エカード配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>緑内障：α２作動+ROCK阻害</t>
+    <rPh sb="0" eb="3">
+      <t>リョクナイショウ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>サドウ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ソガイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>トリクロルメチアジド錠2mg　0.5錠</t>
+    <rPh sb="18" eb="19">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>イルベサルタン錠100mg　１錠</t>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>トリクロルメチアジド１mg</t>
+  </si>
+  <si>
+    <t>イルベサルタン100mg</t>
+  </si>
+  <si>
+    <t>イルトラ配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>緑内障：α２作動+CAI</t>
+    <rPh sb="0" eb="3">
+      <t>リョクナイショウ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>サドウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>イルベサルタン錠100mg　２錠</t>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>イルベサルタン２００mg</t>
+  </si>
+  <si>
+    <t>イルトラ配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>緑内障：α２作動+β遮断</t>
+    <rPh sb="0" eb="3">
+      <t>リョクナイショウ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>サドウ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>シャダン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>イルベサルタン錠100mg　１錠</t>
+    <rPh sb="7" eb="8">
+      <t>ジョウ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>イルアミクス配合錠ＬＤ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>緑内障：CAI+β遮断</t>
+    <rPh sb="0" eb="3">
+      <t>リョクナイショウ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>シャダン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムロジピンOD錠5mg　２錠</t>
+    <rPh sb="14" eb="15">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムロジピン１０mg</t>
+  </si>
+  <si>
+    <t>イルアミクス配合錠HＤ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>緑内障：PG系+β遮断</t>
+    <rPh sb="0" eb="3">
+      <t>リョクナイショウ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>ケイ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>シャダン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アログリプチン２５mg</t>
+  </si>
+  <si>
+    <t>イニシンク配合錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アムバロ配合錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アマルエット配合錠4番</t>
+    <rPh sb="10" eb="11">
+      <t>バン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アマルエット配合錠3番</t>
+    <rPh sb="10" eb="11">
+      <t>バン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アマルエット配合錠2番</t>
+    <rPh sb="10" eb="11">
+      <t>バン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アマルエット配合錠１番</t>
+    <rPh sb="10" eb="11">
+      <t>バン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン１０mg</t>
+  </si>
+  <si>
+    <t>アトーゼット配合錠LD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アトルバスタチン2０mg</t>
+  </si>
+  <si>
+    <t>アトーゼット配合錠HD</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>シルニジピン錠10mg　１錠</t>
+    <rPh sb="13" eb="14">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>シルニジピン１０mg</t>
+  </si>
+  <si>
+    <t>バルサルタン８０mg</t>
+  </si>
+  <si>
+    <t>アテディオ配合錠</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>イルベサルタン錠100mg 1錠</t>
+    <rPh sb="7" eb="8">
+      <t>ジョウ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>ジョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アイミクス配合錠LＤ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>アイミクス配合錠ＨＤ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>列6</t>
+  </si>
+  <si>
+    <t>列5</t>
+  </si>
+  <si>
+    <t>列4</t>
+  </si>
+  <si>
+    <t>列3</t>
+  </si>
+  <si>
+    <t>列2</t>
+  </si>
+  <si>
+    <t>列1</t>
+  </si>
+  <si>
+    <t>分解後商品名②</t>
+    <rPh sb="3" eb="5">
+      <t>ショウヒン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>分解後商品名①</t>
+    <rPh sb="0" eb="2">
+      <t>ブンカイ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ゴ</t>
+    </rPh>
+    <rPh sb="3" eb="6">
+      <t>ショウヒンメイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>分解後成分名②</t>
+    <rPh sb="3" eb="5">
+      <t>セイブン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>分解後成分名①</t>
+    <rPh sb="0" eb="2">
+      <t>ブンカイ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ゴ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>セイブン</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>メイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>当院院内採用薬剤へ変切り替え後</t>
+    <rPh sb="0" eb="2">
+      <t>トウイン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>インナイ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>サイヨウ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ヤクザイ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>ヘン</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>カ</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>ゴ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>分類</t>
+    <rPh sb="0" eb="2">
+      <t>ブンルイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>薬剤名</t>
+    <rPh sb="0" eb="3">
+      <t>ヤクザイメイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>配合錠　当院院内採用薬剤　切り替え一覧表　　2025.10.6</t>
+    <rPh sb="2" eb="3">
+      <t>ジョウ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>トウイン</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>インナイ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>サイヨウ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>ヤクザイ</t>
+    </rPh>
+    <rPh sb="13" eb="14">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>カ</t>
+    </rPh>
+    <rPh sb="17" eb="20">
+      <t>イチランヒョウ</t>
     </rPh>
     <phoneticPr fontId="2"/>
   </si>
@@ -1844,7 +3097,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1881,8 +3134,50 @@
       <family val="3"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1895,8 +3190,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -1919,13 +3220,373 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1962,11 +3623,439 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="HG丸ｺﾞｼｯｸM-PRO"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1977,6 +4066,24 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{634F1065-E033-4FB2-B9DF-0D2F48C63B43}" name="テーブル72" displayName="テーブル72" ref="A5:F106" totalsRowShown="0" headerRowDxfId="7" tableBorderDxfId="6">
+  <autoFilter ref="A5:F106" xr:uid="{A2FD8E97-8A0B-4E79-AC7D-17205FF1138C}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:F106">
+    <sortCondition ref="A6"/>
+  </sortState>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{C9BBA2D8-CDF7-41E7-AD0C-4CCED55287E5}" name="列1" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{41017296-0DBE-4789-9120-093775017507}" name="列2" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{EDB2AA19-3EAD-4105-B981-A244BBA5EC3C}" name="列3" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{6F2E28B0-0B04-4F8B-A270-30ED22A448E6}" name="列4" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C74753C2-41D0-421F-848C-04C8FB873D0A}" name="列5" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{8A062687-734E-47AF-BF85-BD32A669ACDF}" name="列6" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5670,4 +7777,1908 @@
   <pageMargins left="0" right="0" top="0.19685039370078741" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="72" fitToHeight="4" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E818CDDB-3BB4-4594-9EB3-698F54E77174}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H106"/>
+  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <cols>
+    <col min="1" max="1" width="25.625" customWidth="1"/>
+    <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="39.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.7">
+      <c r="A1" s="70" t="s">
+        <v>528</v>
+      </c>
+      <c r="B1" s="70"/>
+    </row>
+    <row r="2" spans="1:8" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.75"/>
+    <row r="3" spans="1:8" s="41" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+      <c r="A3" s="69" t="s">
+        <v>527</v>
+      </c>
+      <c r="B3" s="68" t="s">
+        <v>526</v>
+      </c>
+      <c r="C3" s="67" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" s="66"/>
+      <c r="E3" s="65" t="s">
+        <v>525</v>
+      </c>
+      <c r="F3" s="64"/>
+    </row>
+    <row r="4" spans="1:8" s="41" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+      <c r="A4" s="63"/>
+      <c r="B4" s="62"/>
+      <c r="C4" s="59" t="s">
+        <v>524</v>
+      </c>
+      <c r="D4" s="58" t="s">
+        <v>523</v>
+      </c>
+      <c r="E4" s="57" t="s">
+        <v>522</v>
+      </c>
+      <c r="F4" s="56" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="41" customFormat="1" ht="0.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+      <c r="A5" s="61" t="s">
+        <v>520</v>
+      </c>
+      <c r="B5" s="60" t="s">
+        <v>519</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>518</v>
+      </c>
+      <c r="D5" s="58" t="s">
+        <v>517</v>
+      </c>
+      <c r="E5" s="57" t="s">
+        <v>516</v>
+      </c>
+      <c r="F5" s="56" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A6" s="55" t="s">
+        <v>514</v>
+      </c>
+      <c r="B6" s="54" t="s">
+        <v>321</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>483</v>
+      </c>
+      <c r="D6" s="52" t="s">
+        <v>494</v>
+      </c>
+      <c r="E6" s="51" t="s">
+        <v>512</v>
+      </c>
+      <c r="F6" s="50" t="s">
+        <v>493</v>
+      </c>
+      <c r="H6" s="43" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A7" s="49" t="s">
+        <v>513</v>
+      </c>
+      <c r="B7" s="48" t="s">
+        <v>321</v>
+      </c>
+      <c r="C7" s="47" t="s">
+        <v>483</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>349</v>
+      </c>
+      <c r="E7" s="45" t="s">
+        <v>512</v>
+      </c>
+      <c r="F7" s="44" t="s">
+        <v>376</v>
+      </c>
+      <c r="H7" s="43" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A8" s="42" t="s">
+        <v>511</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>510</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>509</v>
+      </c>
+      <c r="E8" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>508</v>
+      </c>
+      <c r="H8" s="43" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A9" s="35" t="s">
+        <v>507</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>506</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E9" s="31" t="s">
+        <v>469</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>299</v>
+      </c>
+      <c r="H9" s="43" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A10" s="42" t="s">
+        <v>505</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>504</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>447</v>
+      </c>
+      <c r="F10" s="30" t="s">
+        <v>299</v>
+      </c>
+      <c r="H10" s="40" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A11" s="35" t="s">
+        <v>503</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>345</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>453</v>
+      </c>
+      <c r="E11" s="31" t="s">
+        <v>343</v>
+      </c>
+      <c r="F11" s="30" t="s">
+        <v>452</v>
+      </c>
+      <c r="H11" s="40" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A12" s="42" t="s">
+        <v>502</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>345</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>449</v>
+      </c>
+      <c r="E12" s="31" t="s">
+        <v>343</v>
+      </c>
+      <c r="F12" s="30" t="s">
+        <v>447</v>
+      </c>
+      <c r="H12" s="40" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A13" s="35" t="s">
+        <v>501</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>349</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>453</v>
+      </c>
+      <c r="E13" s="31" t="s">
+        <v>448</v>
+      </c>
+      <c r="F13" s="30" t="s">
+        <v>452</v>
+      </c>
+      <c r="H13" s="40" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A14" s="42" t="s">
+        <v>500</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>349</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>449</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>448</v>
+      </c>
+      <c r="F14" s="30" t="s">
+        <v>447</v>
+      </c>
+      <c r="H14" s="40" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A15" s="35" t="s">
+        <v>499</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F15" s="30" t="s">
+        <v>376</v>
+      </c>
+      <c r="H15" s="40" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A16" s="33" t="s">
+        <v>498</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>363</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>497</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>335</v>
+      </c>
+      <c r="H16" s="40" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A17" s="33" t="s">
+        <v>495</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>483</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>494</v>
+      </c>
+      <c r="E17" s="31" t="s">
+        <v>490</v>
+      </c>
+      <c r="F17" s="30" t="s">
+        <v>493</v>
+      </c>
+      <c r="H17" s="40" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A18" s="33" t="s">
+        <v>491</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C18" s="32" t="s">
+        <v>483</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>490</v>
+      </c>
+      <c r="F18" s="30" t="s">
+        <v>376</v>
+      </c>
+      <c r="H18" s="40" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A19" s="33" t="s">
+        <v>488</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C19" s="32" t="s">
+        <v>487</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>482</v>
+      </c>
+      <c r="E19" s="31" t="s">
+        <v>486</v>
+      </c>
+      <c r="F19" s="30" t="s">
+        <v>480</v>
+      </c>
+      <c r="H19" s="40" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" s="41" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A20" s="33" t="s">
+        <v>484</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C20" s="32" t="s">
+        <v>483</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>482</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>481</v>
+      </c>
+      <c r="F20" s="30" t="s">
+        <v>480</v>
+      </c>
+      <c r="H20" s="40" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A21" s="33" t="s">
+        <v>478</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C21" s="32" t="s">
+        <v>460</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="E21" s="31" t="s">
+        <v>344</v>
+      </c>
+      <c r="F21" s="30" t="s">
+        <v>385</v>
+      </c>
+      <c r="H21" s="40" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A22" s="33" t="s">
+        <v>477</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C22" s="32" t="s">
+        <v>458</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="E22" s="31" t="s">
+        <v>457</v>
+      </c>
+      <c r="F22" s="30" t="s">
+        <v>385</v>
+      </c>
+      <c r="H22" s="40" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A23" s="33" t="s">
+        <v>476</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="C23" s="32" t="s">
+        <v>363</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="E23" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="F23" s="30" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A24" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="C24" s="32" t="s">
+        <v>474</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="E24" s="31" t="s">
+        <v>352</v>
+      </c>
+      <c r="F24" s="30" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A25" s="36" t="s">
+        <v>471</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C25" s="32" t="s">
+        <v>470</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E25" s="31" t="s">
+        <v>469</v>
+      </c>
+      <c r="F25" s="30" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A26" s="36" t="s">
+        <v>468</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C26" s="32" t="s">
+        <v>467</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>466</v>
+      </c>
+      <c r="F26" s="30" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A27" s="36" t="s">
+        <v>465</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>303</v>
+      </c>
+      <c r="C27" s="32" t="s">
+        <v>306</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E27" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="F27" s="30" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A28" s="36" t="s">
+        <v>464</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>303</v>
+      </c>
+      <c r="C28" s="32" t="s">
+        <v>463</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>300</v>
+      </c>
+      <c r="F28" s="30" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A29" s="33" t="s">
+        <v>462</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C29" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E29" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F29" s="30" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A30" s="33" t="s">
+        <v>461</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C30" s="32" t="s">
+        <v>460</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="E30" s="31" t="s">
+        <v>344</v>
+      </c>
+      <c r="F30" s="30" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A31" s="33" t="s">
+        <v>459</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C31" s="32" t="s">
+        <v>458</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="E31" s="31" t="s">
+        <v>457</v>
+      </c>
+      <c r="F31" s="30" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A32" s="33" t="s">
+        <v>456</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C32" s="32" t="s">
+        <v>345</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>453</v>
+      </c>
+      <c r="E32" s="31" t="s">
+        <v>343</v>
+      </c>
+      <c r="F32" s="30" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A33" s="33" t="s">
+        <v>455</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C33" s="32" t="s">
+        <v>345</v>
+      </c>
+      <c r="D33" s="17" t="s">
+        <v>449</v>
+      </c>
+      <c r="E33" s="31" t="s">
+        <v>343</v>
+      </c>
+      <c r="F33" s="30" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A34" s="33" t="s">
+        <v>454</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C34" s="32" t="s">
+        <v>349</v>
+      </c>
+      <c r="D34" s="17" t="s">
+        <v>453</v>
+      </c>
+      <c r="E34" s="31" t="s">
+        <v>448</v>
+      </c>
+      <c r="F34" s="30" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A35" s="33" t="s">
+        <v>451</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C35" s="32" t="s">
+        <v>349</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>449</v>
+      </c>
+      <c r="E35" s="31" t="s">
+        <v>448</v>
+      </c>
+      <c r="F35" s="30" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A36" s="33" t="s">
+        <v>446</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="C36" s="32" t="s">
+        <v>445</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>444</v>
+      </c>
+      <c r="E36" s="31" t="s">
+        <v>443</v>
+      </c>
+      <c r="F36" s="30" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A37" s="33" t="s">
+        <v>441</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C37" s="32" t="s">
+        <v>346</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E37" s="31" t="s">
+        <v>344</v>
+      </c>
+      <c r="F37" s="30" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A38" s="33" t="s">
+        <v>440</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C38" s="32" t="s">
+        <v>346</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="E38" s="31" t="s">
+        <v>344</v>
+      </c>
+      <c r="F38" s="30" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A39" s="33" t="s">
+        <v>439</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="C39" s="32" t="s">
+        <v>406</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>438</v>
+      </c>
+      <c r="E39" s="31" t="s">
+        <v>404</v>
+      </c>
+      <c r="F39" s="30" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A40" s="33" t="s">
+        <v>436</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>435</v>
+      </c>
+      <c r="C40" s="32" t="s">
+        <v>434</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>433</v>
+      </c>
+      <c r="E40" s="31" t="s">
+        <v>432</v>
+      </c>
+      <c r="F40" s="30" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A41" s="33" t="s">
+        <v>430</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C41" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="D41" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="E41" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F41" s="30" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A42" s="33" t="s">
+        <v>429</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C42" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="D42" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="E42" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F42" s="30" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A43" s="33" t="s">
+        <v>428</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="C43" s="32" t="s">
+        <v>406</v>
+      </c>
+      <c r="D43" s="17" t="s">
+        <v>427</v>
+      </c>
+      <c r="E43" s="31" t="s">
+        <v>404</v>
+      </c>
+      <c r="F43" s="30" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A44" s="33" t="s">
+        <v>425</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C44" s="32" t="s">
+        <v>421</v>
+      </c>
+      <c r="D44" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E44" s="31" t="s">
+        <v>420</v>
+      </c>
+      <c r="F44" s="30" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A45" s="33" t="s">
+        <v>424</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C45" s="32" t="s">
+        <v>421</v>
+      </c>
+      <c r="D45" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="E45" s="31" t="s">
+        <v>420</v>
+      </c>
+      <c r="F45" s="30" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A46" s="36" t="s">
+        <v>423</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C46" s="32" t="s">
+        <v>421</v>
+      </c>
+      <c r="D46" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E46" s="31" t="s">
+        <v>420</v>
+      </c>
+      <c r="F46" s="30" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A47" s="36" t="s">
+        <v>422</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C47" s="32" t="s">
+        <v>421</v>
+      </c>
+      <c r="D47" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="E47" s="31" t="s">
+        <v>420</v>
+      </c>
+      <c r="F47" s="30" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A48" s="33" t="s">
+        <v>419</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="C48" s="32" t="s">
+        <v>418</v>
+      </c>
+      <c r="D48" s="17" t="s">
+        <v>417</v>
+      </c>
+      <c r="E48" s="31" t="s">
+        <v>416</v>
+      </c>
+      <c r="F48" s="37" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A49" s="33" t="s">
+        <v>415</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="C49" s="32" t="s">
+        <v>341</v>
+      </c>
+      <c r="D49" s="17" t="s">
+        <v>414</v>
+      </c>
+      <c r="E49" s="31" t="s">
+        <v>340</v>
+      </c>
+      <c r="F49" s="30" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A50" s="33" t="s">
+        <v>412</v>
+      </c>
+      <c r="B50" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="C50" s="32" t="s">
+        <v>336</v>
+      </c>
+      <c r="D50" s="17" t="s">
+        <v>410</v>
+      </c>
+      <c r="E50" s="31" t="s">
+        <v>334</v>
+      </c>
+      <c r="F50" s="30" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A51" s="33" t="s">
+        <v>408</v>
+      </c>
+      <c r="B51" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="C51" s="32" t="s">
+        <v>406</v>
+      </c>
+      <c r="D51" s="17" t="s">
+        <v>405</v>
+      </c>
+      <c r="E51" s="31" t="s">
+        <v>404</v>
+      </c>
+      <c r="F51" s="30" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A52" s="33" t="s">
+        <v>402</v>
+      </c>
+      <c r="B52" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C52" s="32" t="s">
+        <v>374</v>
+      </c>
+      <c r="D52" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E52" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="F52" s="30" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A53" s="33" t="s">
+        <v>401</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C53" s="32" t="s">
+        <v>371</v>
+      </c>
+      <c r="D53" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E53" s="31" t="s">
+        <v>369</v>
+      </c>
+      <c r="F53" s="30" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A54" s="33" t="s">
+        <v>400</v>
+      </c>
+      <c r="B54" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C54" s="32" t="s">
+        <v>374</v>
+      </c>
+      <c r="D54" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="E54" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="F54" s="30" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A55" s="33" t="s">
+        <v>399</v>
+      </c>
+      <c r="B55" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C55" s="32" t="s">
+        <v>371</v>
+      </c>
+      <c r="D55" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="E55" s="31" t="s">
+        <v>369</v>
+      </c>
+      <c r="F55" s="30" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A56" s="33" t="s">
+        <v>398</v>
+      </c>
+      <c r="B56" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="C56" s="32" t="s">
+        <v>393</v>
+      </c>
+      <c r="D56" s="17" t="s">
+        <v>397</v>
+      </c>
+      <c r="E56" s="31" t="s">
+        <v>391</v>
+      </c>
+      <c r="F56" s="30" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A57" s="33" t="s">
+        <v>395</v>
+      </c>
+      <c r="B57" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="C57" s="32" t="s">
+        <v>393</v>
+      </c>
+      <c r="D57" s="17" t="s">
+        <v>392</v>
+      </c>
+      <c r="E57" s="31" t="s">
+        <v>391</v>
+      </c>
+      <c r="F57" s="30" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A58" s="33" t="s">
+        <v>389</v>
+      </c>
+      <c r="B58" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C58" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="D58" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="E58" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F58" s="30" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A59" s="33" t="s">
+        <v>388</v>
+      </c>
+      <c r="B59" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C59" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="D59" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="E59" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F59" s="30" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A60" s="33" t="s">
+        <v>384</v>
+      </c>
+      <c r="B60" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C60" s="32" t="s">
+        <v>315</v>
+      </c>
+      <c r="D60" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="E60" s="31" t="s">
+        <v>314</v>
+      </c>
+      <c r="F60" s="30" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A61" s="33" t="s">
+        <v>383</v>
+      </c>
+      <c r="B61" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C61" s="32" t="s">
+        <v>311</v>
+      </c>
+      <c r="D61" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="E61" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="F61" s="30" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A62" s="33" t="s">
+        <v>382</v>
+      </c>
+      <c r="B62" s="18" t="s">
+        <v>381</v>
+      </c>
+      <c r="C62" s="32" t="s">
+        <v>371</v>
+      </c>
+      <c r="D62" s="39" t="s">
+        <v>380</v>
+      </c>
+      <c r="E62" s="31" t="s">
+        <v>369</v>
+      </c>
+      <c r="F62" s="38" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A63" s="33" t="s">
+        <v>378</v>
+      </c>
+      <c r="B63" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C63" s="32" t="s">
+        <v>374</v>
+      </c>
+      <c r="D63" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E63" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="F63" s="30" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A64" s="33" t="s">
+        <v>377</v>
+      </c>
+      <c r="B64" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C64" s="32" t="s">
+        <v>371</v>
+      </c>
+      <c r="D64" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E64" s="31" t="s">
+        <v>369</v>
+      </c>
+      <c r="F64" s="30" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A65" s="33" t="s">
+        <v>375</v>
+      </c>
+      <c r="B65" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C65" s="32" t="s">
+        <v>374</v>
+      </c>
+      <c r="D65" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="E65" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="F65" s="30" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A66" s="33" t="s">
+        <v>372</v>
+      </c>
+      <c r="B66" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C66" s="32" t="s">
+        <v>371</v>
+      </c>
+      <c r="D66" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="E66" s="31" t="s">
+        <v>369</v>
+      </c>
+      <c r="F66" s="30" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A67" s="33" t="s">
+        <v>367</v>
+      </c>
+      <c r="B67" s="18" t="s">
+        <v>365</v>
+      </c>
+      <c r="C67" s="32" t="s">
+        <v>363</v>
+      </c>
+      <c r="D67" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="E67" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="F67" s="30" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A68" s="33" t="s">
+        <v>366</v>
+      </c>
+      <c r="B68" s="18" t="s">
+        <v>365</v>
+      </c>
+      <c r="C68" s="32" t="s">
+        <v>363</v>
+      </c>
+      <c r="D68" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="E68" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="F68" s="30" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A69" s="33" t="s">
+        <v>364</v>
+      </c>
+      <c r="B69" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="C69" s="32" t="s">
+        <v>363</v>
+      </c>
+      <c r="D69" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="E69" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="F69" s="37" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A70" s="33" t="s">
+        <v>362</v>
+      </c>
+      <c r="B70" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="C70" s="32" t="s">
+        <v>354</v>
+      </c>
+      <c r="D70" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="E70" s="31" t="s">
+        <v>352</v>
+      </c>
+      <c r="F70" s="37" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A71" s="36" t="s">
+        <v>360</v>
+      </c>
+      <c r="B71" s="23" t="s">
+        <v>355</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>359</v>
+      </c>
+      <c r="D71" s="23" t="s">
+        <v>353</v>
+      </c>
+      <c r="E71" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="F71" s="35" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A72" s="36" t="s">
+        <v>356</v>
+      </c>
+      <c r="B72" s="23" t="s">
+        <v>355</v>
+      </c>
+      <c r="C72" s="19" t="s">
+        <v>354</v>
+      </c>
+      <c r="D72" s="23" t="s">
+        <v>353</v>
+      </c>
+      <c r="E72" s="31" t="s">
+        <v>352</v>
+      </c>
+      <c r="F72" s="35" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A73" s="33" t="s">
+        <v>350</v>
+      </c>
+      <c r="B73" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C73" s="32" t="s">
+        <v>346</v>
+      </c>
+      <c r="D73" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E73" s="31" t="s">
+        <v>344</v>
+      </c>
+      <c r="F73" s="30" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A74" s="35" t="s">
+        <v>347</v>
+      </c>
+      <c r="B74" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C74" s="32" t="s">
+        <v>346</v>
+      </c>
+      <c r="D74" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="E74" s="31" t="s">
+        <v>344</v>
+      </c>
+      <c r="F74" s="30" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A75" s="33" t="s">
+        <v>342</v>
+      </c>
+      <c r="B75" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="C75" s="32" t="s">
+        <v>337</v>
+      </c>
+      <c r="D75" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="E75" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F75" s="30" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A76" s="33" t="s">
+        <v>339</v>
+      </c>
+      <c r="B76" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="C76" s="32" t="s">
+        <v>337</v>
+      </c>
+      <c r="D76" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="E76" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="F76" s="30" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A77" s="33" t="s">
+        <v>333</v>
+      </c>
+      <c r="B77" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C77" s="32" t="s">
+        <v>332</v>
+      </c>
+      <c r="D77" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E77" s="31" t="s">
+        <v>331</v>
+      </c>
+      <c r="F77" s="30" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A78" s="33" t="s">
+        <v>330</v>
+      </c>
+      <c r="B78" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C78" s="32" t="s">
+        <v>329</v>
+      </c>
+      <c r="D78" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E78" s="31" t="s">
+        <v>328</v>
+      </c>
+      <c r="F78" s="30" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A79" s="33" t="s">
+        <v>327</v>
+      </c>
+      <c r="B79" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C79" s="32" t="s">
+        <v>326</v>
+      </c>
+      <c r="D79" s="17" t="s">
+        <v>325</v>
+      </c>
+      <c r="E79" s="31" t="s">
+        <v>324</v>
+      </c>
+      <c r="F79" s="30" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A80" s="33" t="s">
+        <v>322</v>
+      </c>
+      <c r="B80" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C80" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="D80" s="17" t="s">
+        <v>319</v>
+      </c>
+      <c r="E80" s="31" t="s">
+        <v>318</v>
+      </c>
+      <c r="F80" s="30" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A81" s="33" t="s">
+        <v>316</v>
+      </c>
+      <c r="B81" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C81" s="32" t="s">
+        <v>315</v>
+      </c>
+      <c r="D81" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="E81" s="31" t="s">
+        <v>314</v>
+      </c>
+      <c r="F81" s="30" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A82" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="B82" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C82" s="32" t="s">
+        <v>311</v>
+      </c>
+      <c r="D82" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="E82" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="F82" s="30" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A83" s="33" t="s">
+        <v>307</v>
+      </c>
+      <c r="B83" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="C83" s="32" t="s">
+        <v>306</v>
+      </c>
+      <c r="D83" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="E83" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="F83" s="30" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+      <c r="A84" s="29" t="s">
+        <v>304</v>
+      </c>
+      <c r="B84" s="28" t="s">
+        <v>303</v>
+      </c>
+      <c r="C84" s="27" t="s">
+        <v>302</v>
+      </c>
+      <c r="D84" s="26" t="s">
+        <v>301</v>
+      </c>
+      <c r="E84" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="F84" s="24" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A85" s="21"/>
+      <c r="B85" s="20"/>
+      <c r="C85" s="21"/>
+      <c r="D85" s="23"/>
+      <c r="E85" s="23"/>
+      <c r="F85" s="22"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A86" s="16"/>
+      <c r="B86" s="15"/>
+      <c r="C86" s="14"/>
+      <c r="D86" s="13"/>
+      <c r="E86" s="13"/>
+      <c r="F86" s="12"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A87" s="21"/>
+      <c r="B87" s="20"/>
+      <c r="C87" s="19"/>
+      <c r="D87" s="18"/>
+      <c r="E87" s="18"/>
+      <c r="F87" s="17"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A88" s="16"/>
+      <c r="B88" s="15"/>
+      <c r="C88" s="14"/>
+      <c r="D88" s="13"/>
+      <c r="E88" s="13"/>
+      <c r="F88" s="12"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A89" s="21"/>
+      <c r="B89" s="20"/>
+      <c r="C89" s="19"/>
+      <c r="D89" s="18"/>
+      <c r="E89" s="18"/>
+      <c r="F89" s="17"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A90" s="16"/>
+      <c r="B90" s="15"/>
+      <c r="C90" s="14"/>
+      <c r="D90" s="13"/>
+      <c r="E90" s="13"/>
+      <c r="F90" s="12"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A91" s="21"/>
+      <c r="B91" s="20"/>
+      <c r="C91" s="19"/>
+      <c r="D91" s="18"/>
+      <c r="E91" s="18"/>
+      <c r="F91" s="17"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A92" s="16"/>
+      <c r="B92" s="15"/>
+      <c r="C92" s="14"/>
+      <c r="D92" s="13"/>
+      <c r="E92" s="13"/>
+      <c r="F92" s="12"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A93" s="16"/>
+      <c r="B93" s="15"/>
+      <c r="C93" s="14"/>
+      <c r="D93" s="13"/>
+      <c r="E93" s="13"/>
+      <c r="F93" s="12"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A94" s="16"/>
+      <c r="B94" s="15"/>
+      <c r="C94" s="14"/>
+      <c r="D94" s="13"/>
+      <c r="E94" s="13"/>
+      <c r="F94" s="12"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A95" s="16"/>
+      <c r="B95" s="15"/>
+      <c r="C95" s="14"/>
+      <c r="D95" s="13"/>
+      <c r="E95" s="13"/>
+      <c r="F95" s="12"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A96" s="16"/>
+      <c r="B96" s="15"/>
+      <c r="C96" s="14"/>
+      <c r="D96" s="13"/>
+      <c r="E96" s="13"/>
+      <c r="F96" s="12"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A97" s="16"/>
+      <c r="B97" s="15"/>
+      <c r="C97" s="14"/>
+      <c r="D97" s="13"/>
+      <c r="E97" s="13"/>
+      <c r="F97" s="12"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A98" s="16"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="14"/>
+      <c r="D98" s="13"/>
+      <c r="E98" s="13"/>
+      <c r="F98" s="12"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A99" s="16"/>
+      <c r="B99" s="15"/>
+      <c r="C99" s="14"/>
+      <c r="D99" s="13"/>
+      <c r="E99" s="13"/>
+      <c r="F99" s="12"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A100" s="16"/>
+      <c r="B100" s="15"/>
+      <c r="C100" s="14"/>
+      <c r="D100" s="13"/>
+      <c r="E100" s="13"/>
+      <c r="F100" s="12"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A101" s="16"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="14"/>
+      <c r="D101" s="13"/>
+      <c r="E101" s="13"/>
+      <c r="F101" s="12"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A102" s="16"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="14"/>
+      <c r="D102" s="13"/>
+      <c r="E102" s="13"/>
+      <c r="F102" s="12"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A103" s="16"/>
+      <c r="B103" s="15"/>
+      <c r="C103" s="14"/>
+      <c r="D103" s="13"/>
+      <c r="E103" s="13"/>
+      <c r="F103" s="12"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A104" s="16"/>
+      <c r="B104" s="15"/>
+      <c r="C104" s="14"/>
+      <c r="D104" s="13"/>
+      <c r="E104" s="13"/>
+      <c r="F104" s="12"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A105" s="16"/>
+      <c r="B105" s="15"/>
+      <c r="C105" s="14"/>
+      <c r="D105" s="13"/>
+      <c r="E105" s="13"/>
+      <c r="F105" s="12"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.7">
+      <c r="A106" s="16"/>
+      <c r="B106" s="15"/>
+      <c r="C106" s="14"/>
+      <c r="D106" s="13"/>
+      <c r="E106" s="13"/>
+      <c r="F106" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+  </mergeCells>
+  <phoneticPr fontId="2"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6:B106" xr:uid="{70FF8F1A-3FCC-426F-9EB8-61BF7A45D1B6}">
+      <formula1>$H$6:$H$23</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.70866141732283472" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="47" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>